<commit_message>
Extend date range by one trailing day, carrying forward last day's qty
excel_format_conversion.py now adds one extra date column after the
last real date column (e.g. last date 7/3 -> also emit 7/4), reusing
the last date's quantity for every category. Configurable via
--extend-days (default 1, 0 disables). Regenerated the committed
CategorySIPMaintain.7.3.long.xlsx with this change (7/4-7/11, 232 rows).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.3.long.xlsx
+++ b/CategorySIPMaintain.7.3.long.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4081,6 +4081,524 @@
         <v>80</v>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C205" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D205" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>T59B</t>
+        </is>
+      </c>
+      <c r="C206" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D206" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>T59B 2</t>
+        </is>
+      </c>
+      <c r="C207" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>T528B</t>
+        </is>
+      </c>
+      <c r="C208" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D208" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C209" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D209" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Flat T</t>
+        </is>
+      </c>
+      <c r="C210" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D210" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>T-A42</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D211" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>T-G</t>
+        </is>
+      </c>
+      <c r="C212" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D212" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>T523T</t>
+        </is>
+      </c>
+      <c r="C213" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D213" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C215" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C216" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D216" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1.9V</t>
+        </is>
+      </c>
+      <c r="C217" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D217" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2.0V</t>
+        </is>
+      </c>
+      <c r="C218" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D218" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D219" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D220" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C221" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D221" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>T530D 2</t>
+        </is>
+      </c>
+      <c r="C222" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D222" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>T530D 3</t>
+        </is>
+      </c>
+      <c r="C223" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D223" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>T530X</t>
+        </is>
+      </c>
+      <c r="C224" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D224" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>T521X</t>
+        </is>
+      </c>
+      <c r="C225" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D225" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>T530Y</t>
+        </is>
+      </c>
+      <c r="C226" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D226" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>T59D 2</t>
+        </is>
+      </c>
+      <c r="C227" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D227" t="n">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>T59D 1</t>
+        </is>
+      </c>
+      <c r="C228" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D228" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>T59V</t>
+        </is>
+      </c>
+      <c r="C229" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D229" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>T528Z 1</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D230" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>T523W</t>
+        </is>
+      </c>
+      <c r="C231" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D231" t="n">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>T528Z 2</t>
+        </is>
+      </c>
+      <c r="C232" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D232" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>T523H</t>
+        </is>
+      </c>
+      <c r="C233" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="D233" t="n">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Drop rows with a zero or blank Quantity from the output
excel_format_conversion.py now filters out rows whose Quantity is 0 or
NaN before writing the long-format sheet. Regenerated
CategorySIPMaintain.7.3.long.xlsx accordingly (232 -> 179 rows).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.3.long.xlsx
+++ b/CategorySIPMaintain.7.3.long.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D233"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -493,13 +493,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
         <v>46207</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -509,14 +511,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -527,14 +529,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D6" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -545,14 +547,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D7" t="n">
-        <v>84</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8">
@@ -563,14 +565,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C8" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D8" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="9">
@@ -581,14 +583,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C9" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D9" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -599,14 +601,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -617,14 +619,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
@@ -635,13 +637,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
         <v>46207</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -651,14 +655,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D13" t="n">
-        <v>900</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -669,14 +673,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D14" t="n">
-        <v>120</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15">
@@ -687,14 +691,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D15" t="n">
-        <v>150</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16">
@@ -705,14 +709,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17">
@@ -723,14 +727,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18">
@@ -741,14 +745,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C18" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D18" t="n">
-        <v>10</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19">
@@ -759,14 +763,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C19" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D19" t="n">
-        <v>84</v>
+        <v>630</v>
       </c>
     </row>
     <row r="20">
@@ -777,14 +781,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D20" t="n">
-        <v>168</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21">
@@ -795,14 +799,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C21" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D21" t="n">
-        <v>200</v>
+        <v>420</v>
       </c>
     </row>
     <row r="22">
@@ -813,14 +817,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C22" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D22" t="n">
-        <v>90</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23">
@@ -831,14 +835,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
         <v>46207</v>
       </c>
       <c r="D23" t="n">
-        <v>174</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
@@ -849,14 +853,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D24" t="n">
-        <v>630</v>
+        <v>850</v>
       </c>
     </row>
     <row r="25">
@@ -867,14 +871,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D25" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
@@ -885,14 +889,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D26" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="27">
@@ -903,14 +907,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28">
@@ -921,14 +925,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D28" t="n">
-        <v>322</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29">
@@ -939,14 +943,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C29" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30">
@@ -957,14 +961,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="D30" t="n">
-        <v>80</v>
+        <v>900</v>
       </c>
     </row>
     <row r="31">
@@ -975,14 +979,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D31" t="n">
-        <v>850</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32">
@@ -993,7 +997,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
@@ -1011,13 +1015,15 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
         <v>46208</v>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1027,14 +1033,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -1045,14 +1051,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C35" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D35" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36">
@@ -1063,7 +1069,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C36" s="1" t="n">
@@ -1081,14 +1087,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C37" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D37" t="n">
-        <v>1000</v>
+        <v>168</v>
       </c>
     </row>
     <row r="38">
@@ -1099,14 +1105,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C38" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D38" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="39">
@@ -1117,14 +1123,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C39" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40">
@@ -1135,14 +1141,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C40" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
     </row>
     <row r="41">
@@ -1153,13 +1159,15 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C41" s="1" t="n">
         <v>46208</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="n">
+        <v>630</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1169,14 +1177,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C42" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D42" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43">
@@ -1187,14 +1195,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C43" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D43" t="n">
-        <v>120</v>
+        <v>420</v>
       </c>
     </row>
     <row r="44">
@@ -1205,14 +1213,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C44" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D44" t="n">
-        <v>150</v>
+        <v>322</v>
       </c>
     </row>
     <row r="45">
@@ -1223,14 +1231,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C45" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D45" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46">
@@ -1241,14 +1249,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C46" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D46" t="n">
-        <v>20</v>
+        <v>850</v>
       </c>
     </row>
     <row r="47">
@@ -1259,14 +1267,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C47" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D47" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
     </row>
     <row r="48">
@@ -1277,14 +1285,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C48" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D48" t="n">
-        <v>84</v>
+        <v>200</v>
       </c>
     </row>
     <row r="49">
@@ -1295,14 +1303,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C49" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D49" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50">
@@ -1313,14 +1321,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C50" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D50" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="51">
@@ -1331,14 +1339,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C51" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D51" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="52">
@@ -1349,14 +1357,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C52" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D52" t="n">
-        <v>174</v>
+        <v>900</v>
       </c>
     </row>
     <row r="53">
@@ -1367,14 +1375,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C53" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D53" t="n">
-        <v>630</v>
+        <v>120</v>
       </c>
     </row>
     <row r="54">
@@ -1385,14 +1393,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C54" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D54" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="55">
@@ -1403,14 +1411,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C55" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D55" t="n">
-        <v>420</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56">
@@ -1421,14 +1429,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C56" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57">
@@ -1439,14 +1447,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C57" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D57" t="n">
-        <v>322</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58">
@@ -1457,14 +1465,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C58" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59">
@@ -1475,14 +1483,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C59" s="1" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="D59" t="n">
-        <v>80</v>
+        <v>168</v>
       </c>
     </row>
     <row r="60">
@@ -1493,14 +1501,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C60" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D60" t="n">
-        <v>850</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61">
@@ -1511,14 +1519,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C61" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D61" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62">
@@ -1529,13 +1537,15 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C62" s="1" t="n">
         <v>46209</v>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="n">
+        <v>174</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1545,14 +1555,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C63" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>630</v>
       </c>
     </row>
     <row r="64">
@@ -1563,7 +1573,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C64" s="1" t="n">
@@ -1581,14 +1591,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C65" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D65" t="n">
-        <v>84</v>
+        <v>420</v>
       </c>
     </row>
     <row r="66">
@@ -1599,14 +1609,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C66" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D66" t="n">
-        <v>1000</v>
+        <v>322</v>
       </c>
     </row>
     <row r="67">
@@ -1617,14 +1627,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C67" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D67" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
     </row>
     <row r="68">
@@ -1635,14 +1645,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C68" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>850</v>
       </c>
     </row>
     <row r="69">
@@ -1653,14 +1663,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C69" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="70">
@@ -1671,13 +1681,15 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C70" s="1" t="n">
-        <v>46209</v>
-      </c>
-      <c r="D70" t="inlineStr"/>
+        <v>46210</v>
+      </c>
+      <c r="D70" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1687,14 +1699,14 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C71" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D71" t="n">
-        <v>900</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72">
@@ -1705,14 +1717,14 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C72" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D72" t="n">
-        <v>120</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="73">
@@ -1723,11 +1735,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C73" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D73" t="n">
         <v>150</v>
@@ -1741,14 +1753,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C74" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D74" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="75">
@@ -1759,14 +1771,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C75" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D75" t="n">
-        <v>20</v>
+        <v>900</v>
       </c>
     </row>
     <row r="76">
@@ -1777,14 +1789,14 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C76" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D76" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77">
@@ -1795,14 +1807,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C77" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>150</v>
       </c>
     </row>
     <row r="78">
@@ -1813,14 +1825,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C78" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D78" t="n">
-        <v>168</v>
+        <v>60</v>
       </c>
     </row>
     <row r="79">
@@ -1831,14 +1843,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C79" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D79" t="n">
-        <v>200</v>
+        <v>20</v>
       </c>
     </row>
     <row r="80">
@@ -1849,14 +1861,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C80" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D80" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81">
@@ -1867,14 +1879,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C81" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D81" t="n">
-        <v>174</v>
+        <v>84</v>
       </c>
     </row>
     <row r="82">
@@ -1885,14 +1897,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C82" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D82" t="n">
-        <v>630</v>
+        <v>168</v>
       </c>
     </row>
     <row r="83">
@@ -1903,11 +1915,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C83" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D83" t="n">
         <v>200</v>
@@ -1921,14 +1933,14 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C84" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D84" t="n">
-        <v>420</v>
+        <v>90</v>
       </c>
     </row>
     <row r="85">
@@ -1939,14 +1951,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C85" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
     </row>
     <row r="86">
@@ -1957,14 +1969,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C86" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D86" t="n">
-        <v>322</v>
+        <v>630</v>
       </c>
     </row>
     <row r="87">
@@ -1975,14 +1987,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C87" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="88">
@@ -1993,14 +2005,14 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C88" s="1" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="D88" t="n">
-        <v>80</v>
+        <v>420</v>
       </c>
     </row>
     <row r="89">
@@ -2011,14 +2023,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C89" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D89" t="n">
-        <v>850</v>
+        <v>322</v>
       </c>
     </row>
     <row r="90">
@@ -2029,14 +2041,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C90" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D90" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
     </row>
     <row r="91">
@@ -2047,13 +2059,15 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C91" s="1" t="n">
-        <v>46210</v>
-      </c>
-      <c r="D91" t="inlineStr"/>
+        <v>46211</v>
+      </c>
+      <c r="D91" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2063,14 +2077,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C92" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="93">
@@ -2081,14 +2095,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B 2</t>
         </is>
       </c>
       <c r="C93" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D93" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94">
@@ -2099,14 +2113,14 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C94" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D94" t="n">
-        <v>84</v>
+        <v>350</v>
       </c>
     </row>
     <row r="95">
@@ -2117,14 +2131,14 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C95" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D95" t="n">
-        <v>1050</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96">
@@ -2135,14 +2149,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C96" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D96" t="n">
-        <v>150</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="97">
@@ -2153,14 +2167,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C97" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="98">
@@ -2171,14 +2185,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C98" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="99">
@@ -2189,14 +2203,14 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C99" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D99" t="n">
-        <v>66</v>
+        <v>120</v>
       </c>
     </row>
     <row r="100">
@@ -2207,14 +2221,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C100" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D100" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="101">
@@ -2225,14 +2239,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C101" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D101" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="102">
@@ -2243,14 +2257,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C102" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D102" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
     </row>
     <row r="103">
@@ -2261,14 +2275,14 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C103" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D103" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104">
@@ -2279,14 +2293,14 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C104" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D104" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
     </row>
     <row r="105">
@@ -2297,14 +2311,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C105" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>168</v>
       </c>
     </row>
     <row r="106">
@@ -2315,14 +2329,14 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C106" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D106" t="n">
-        <v>84</v>
+        <v>200</v>
       </c>
     </row>
     <row r="107">
@@ -2333,14 +2347,14 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C107" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D107" t="n">
-        <v>168</v>
+        <v>90</v>
       </c>
     </row>
     <row r="108">
@@ -2351,14 +2365,14 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C108" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D108" t="n">
-        <v>200</v>
+        <v>174</v>
       </c>
     </row>
     <row r="109">
@@ -2369,14 +2383,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C109" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D109" t="n">
-        <v>90</v>
+        <v>630</v>
       </c>
     </row>
     <row r="110">
@@ -2387,14 +2401,14 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C110" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D110" t="n">
-        <v>174</v>
+        <v>200</v>
       </c>
     </row>
     <row r="111">
@@ -2405,14 +2419,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C111" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D111" t="n">
-        <v>630</v>
+        <v>420</v>
       </c>
     </row>
     <row r="112">
@@ -2423,14 +2437,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C112" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D112" t="n">
-        <v>200</v>
+        <v>322</v>
       </c>
     </row>
     <row r="113">
@@ -2441,14 +2455,14 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C113" s="1" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D113" t="n">
-        <v>420</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114">
@@ -2459,14 +2473,14 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C114" s="1" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="115">
@@ -2477,14 +2491,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C115" s="1" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="D115" t="n">
-        <v>322</v>
+        <v>150</v>
       </c>
     </row>
     <row r="116">
@@ -2495,14 +2509,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>T59B 2</t>
         </is>
       </c>
       <c r="C116" s="1" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="D116" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="117">
@@ -2513,14 +2527,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C117" s="1" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="D117" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
     </row>
     <row r="118">
@@ -2531,14 +2545,14 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C118" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D118" t="n">
-        <v>650</v>
+        <v>84</v>
       </c>
     </row>
     <row r="119">
@@ -2549,14 +2563,14 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C119" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D119" t="n">
-        <v>150</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="120">
@@ -2567,14 +2581,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C120" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D120" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
     </row>
     <row r="121">
@@ -2585,14 +2599,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C121" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="122">
@@ -2603,14 +2617,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C122" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D122" t="n">
-        <v>350</v>
+        <v>120</v>
       </c>
     </row>
     <row r="123">
@@ -2621,14 +2635,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C123" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D123" t="n">
-        <v>84</v>
+        <v>150</v>
       </c>
     </row>
     <row r="124">
@@ -2639,14 +2653,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C124" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D124" t="n">
-        <v>1050</v>
+        <v>60</v>
       </c>
     </row>
     <row r="125">
@@ -2657,14 +2671,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C125" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D125" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
     </row>
     <row r="126">
@@ -2675,14 +2689,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C126" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D126" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127">
@@ -2693,14 +2707,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C127" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D127" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="128">
@@ -2711,13 +2725,15 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C128" s="1" t="n">
-        <v>46211</v>
-      </c>
-      <c r="D128" t="inlineStr"/>
+        <v>46212</v>
+      </c>
+      <c r="D128" t="n">
+        <v>168</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2727,14 +2743,14 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C129" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D129" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
     </row>
     <row r="130">
@@ -2745,14 +2761,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C130" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D130" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="131">
@@ -2763,14 +2779,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C131" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D131" t="n">
-        <v>150</v>
+        <v>174</v>
       </c>
     </row>
     <row r="132">
@@ -2781,14 +2797,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C132" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D132" t="n">
-        <v>60</v>
+        <v>630</v>
       </c>
     </row>
     <row r="133">
@@ -2799,14 +2815,14 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C133" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D133" t="n">
-        <v>20</v>
+        <v>200</v>
       </c>
     </row>
     <row r="134">
@@ -2817,14 +2833,14 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C134" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D134" t="n">
-        <v>10</v>
+        <v>420</v>
       </c>
     </row>
     <row r="135">
@@ -2835,14 +2851,14 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C135" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>322</v>
       </c>
     </row>
     <row r="136">
@@ -2853,14 +2869,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C136" s="1" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D136" t="n">
-        <v>168</v>
+        <v>80</v>
       </c>
     </row>
     <row r="137">
@@ -2871,14 +2887,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C137" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D137" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
     </row>
     <row r="138">
@@ -2889,14 +2905,14 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C138" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D138" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="139">
@@ -2907,14 +2923,14 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C139" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D139" t="n">
-        <v>174</v>
+        <v>400</v>
       </c>
     </row>
     <row r="140">
@@ -2925,14 +2941,14 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C140" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D140" t="n">
-        <v>630</v>
+        <v>84</v>
       </c>
     </row>
     <row r="141">
@@ -2943,14 +2959,14 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C141" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D141" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="142">
@@ -2961,14 +2977,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C142" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D142" t="n">
-        <v>420</v>
+        <v>150</v>
       </c>
     </row>
     <row r="143">
@@ -2979,14 +2995,14 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C143" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="144">
@@ -2997,14 +3013,14 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C144" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D144" t="n">
-        <v>322</v>
+        <v>120</v>
       </c>
     </row>
     <row r="145">
@@ -3015,14 +3031,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C145" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D145" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="146">
@@ -3033,14 +3049,14 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C146" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="D146" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="147">
@@ -3051,14 +3067,14 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C147" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D147" t="n">
-        <v>600</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148">
@@ -3069,14 +3085,14 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C148" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D148" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
     </row>
     <row r="149">
@@ -3087,14 +3103,14 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C149" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D149" t="n">
-        <v>150</v>
+        <v>84</v>
       </c>
     </row>
     <row r="150">
@@ -3105,14 +3121,14 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C150" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D150" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
     </row>
     <row r="151">
@@ -3123,14 +3139,14 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C151" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D151" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
     </row>
     <row r="152">
@@ -3141,14 +3157,14 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C152" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D152" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="153">
@@ -3159,14 +3175,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C153" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D153" t="n">
-        <v>1050</v>
+        <v>174</v>
       </c>
     </row>
     <row r="154">
@@ -3177,14 +3193,14 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C154" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D154" t="n">
-        <v>150</v>
+        <v>630</v>
       </c>
     </row>
     <row r="155">
@@ -3195,14 +3211,14 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>T523T</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C155" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D155" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="156">
@@ -3213,14 +3229,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C156" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
     </row>
     <row r="157">
@@ -3231,13 +3247,15 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C157" s="1" t="n">
-        <v>46212</v>
-      </c>
-      <c r="D157" t="inlineStr"/>
+        <v>46213</v>
+      </c>
+      <c r="D157" t="n">
+        <v>322</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3247,14 +3265,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C158" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D158" t="n">
-        <v>900</v>
+        <v>80</v>
       </c>
     </row>
     <row r="159">
@@ -3265,14 +3283,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C159" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D159" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
     </row>
     <row r="160">
@@ -3283,11 +3301,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C160" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D160" t="n">
         <v>150</v>
@@ -3301,14 +3319,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C161" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D161" t="n">
-        <v>60</v>
+        <v>400</v>
       </c>
     </row>
     <row r="162">
@@ -3319,14 +3337,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C162" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D162" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
     </row>
     <row r="163">
@@ -3337,14 +3355,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C163" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D163" t="n">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="164">
@@ -3355,14 +3373,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C164" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D164" t="n">
-        <v>84</v>
+        <v>150</v>
       </c>
     </row>
     <row r="165">
@@ -3373,14 +3391,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C165" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D165" t="n">
-        <v>168</v>
+        <v>900</v>
       </c>
     </row>
     <row r="166">
@@ -3391,14 +3409,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C166" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D166" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
     </row>
     <row r="167">
@@ -3409,14 +3427,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C167" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D167" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="168">
@@ -3427,14 +3445,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C168" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D168" t="n">
-        <v>174</v>
+        <v>60</v>
       </c>
     </row>
     <row r="169">
@@ -3445,14 +3463,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C169" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D169" t="n">
-        <v>630</v>
+        <v>20</v>
       </c>
     </row>
     <row r="170">
@@ -3463,14 +3481,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C170" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D170" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171">
@@ -3481,14 +3499,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C171" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D171" t="n">
-        <v>420</v>
+        <v>84</v>
       </c>
     </row>
     <row r="172">
@@ -3499,14 +3517,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>T528Z 1</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C172" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D172" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
     </row>
     <row r="173">
@@ -3517,14 +3535,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C173" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D173" t="n">
-        <v>322</v>
+        <v>200</v>
       </c>
     </row>
     <row r="174">
@@ -3535,14 +3553,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>T528Z 2</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C174" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D174" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="175">
@@ -3553,14 +3571,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C175" s="1" t="n">
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="D175" t="n">
-        <v>80</v>
+        <v>174</v>
       </c>
     </row>
     <row r="176">
@@ -3571,14 +3589,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C176" s="1" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D176" t="n">
-        <v>600</v>
+        <v>630</v>
       </c>
     </row>
     <row r="177">
@@ -3589,14 +3607,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C177" s="1" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D177" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="178">
@@ -3607,13 +3625,15 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C178" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D178" t="inlineStr"/>
+        <v>46214</v>
+      </c>
+      <c r="D178" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3623,14 +3643,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C179" s="1" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D179" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
     </row>
     <row r="180">
@@ -3641,961 +3661,13 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C180" s="1" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="D180" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Flat T</t>
-        </is>
-      </c>
-      <c r="C181" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D181" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>T-A42</t>
-        </is>
-      </c>
-      <c r="C182" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D182" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>T-G</t>
-        </is>
-      </c>
-      <c r="C183" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D183" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>T523T</t>
-        </is>
-      </c>
-      <c r="C184" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D184" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C185" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D185" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="C186" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D186" t="inlineStr"/>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C187" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D187" t="n">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>1.9V</t>
-        </is>
-      </c>
-      <c r="C188" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D188" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>2.0V</t>
-        </is>
-      </c>
-      <c r="C189" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D189" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="C190" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D190" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C191" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D191" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C192" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D192" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>T530D 2</t>
-        </is>
-      </c>
-      <c r="C193" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D193" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>T530D 3</t>
-        </is>
-      </c>
-      <c r="C194" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D194" t="n">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>T530X</t>
-        </is>
-      </c>
-      <c r="C195" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D195" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>T521X</t>
-        </is>
-      </c>
-      <c r="C196" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D196" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>T530Y</t>
-        </is>
-      </c>
-      <c r="C197" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D197" t="n">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>T59D 2</t>
-        </is>
-      </c>
-      <c r="C198" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D198" t="n">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>T59D 1</t>
-        </is>
-      </c>
-      <c r="C199" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D199" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>T59V</t>
-        </is>
-      </c>
-      <c r="C200" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D200" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>T528Z 1</t>
-        </is>
-      </c>
-      <c r="C201" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D201" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>T523W</t>
-        </is>
-      </c>
-      <c r="C202" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D202" t="n">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>T528Z 2</t>
-        </is>
-      </c>
-      <c r="C203" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D203" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>T523H</t>
-        </is>
-      </c>
-      <c r="C204" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="D204" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C205" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D205" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>T59B</t>
-        </is>
-      </c>
-      <c r="C206" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D206" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>T59B 2</t>
-        </is>
-      </c>
-      <c r="C207" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D207" t="inlineStr"/>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>T528B</t>
-        </is>
-      </c>
-      <c r="C208" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D208" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C209" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D209" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>Flat T</t>
-        </is>
-      </c>
-      <c r="C210" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D210" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>T-A42</t>
-        </is>
-      </c>
-      <c r="C211" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D211" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>T-G</t>
-        </is>
-      </c>
-      <c r="C212" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D212" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>T523T</t>
-        </is>
-      </c>
-      <c r="C213" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D213" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C214" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D214" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="C215" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D215" t="inlineStr"/>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C216" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D216" t="n">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>1.9V</t>
-        </is>
-      </c>
-      <c r="C217" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D217" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>2.0V</t>
-        </is>
-      </c>
-      <c r="C218" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D218" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="C219" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D219" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C220" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D220" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C221" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D221" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>T530D 2</t>
-        </is>
-      </c>
-      <c r="C222" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D222" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>T530D 3</t>
-        </is>
-      </c>
-      <c r="C223" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D223" t="n">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>T530X</t>
-        </is>
-      </c>
-      <c r="C224" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D224" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>T521X</t>
-        </is>
-      </c>
-      <c r="C225" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D225" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>T530Y</t>
-        </is>
-      </c>
-      <c r="C226" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D226" t="n">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>T59D 2</t>
-        </is>
-      </c>
-      <c r="C227" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D227" t="n">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>T59D 1</t>
-        </is>
-      </c>
-      <c r="C228" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D228" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>T59V</t>
-        </is>
-      </c>
-      <c r="C229" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D229" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>T528Z 1</t>
-        </is>
-      </c>
-      <c r="C230" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D230" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>T523W</t>
-        </is>
-      </c>
-      <c r="C231" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D231" t="n">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>T528Z 2</t>
-        </is>
-      </c>
-      <c r="C232" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D232" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>T523H</t>
-        </is>
-      </c>
-      <c r="C233" s="1" t="n">
-        <v>46214</v>
-      </c>
-      <c r="D233" t="n">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Flag earliest-date rows as UPDATE when they differ from a reference
Add --reference: a (Category, quantity) sheet holding already-known
quantities for the earliest date in the output. For that date's rows
only, if the reference quantity is non-zero and differs from the
computed Quantity, UploadType is changed to UPDATE (categories missing
from the reference, or where the reference is 0, stay ADD). Other
dates are untouched.

Regenerated CategorySIPMaintain.7.3.long.xlsx against
CategorySIPMaintain (1).xlsx as the reference - 4 rows on 7/4 flagged
as UPDATE (T59B, 2.0V, X, T530Y).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.3.long.xlsx
+++ b/CategorySIPMaintain.7.3.long.xlsx
@@ -470,7 +470,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>UPDATE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>UPDATE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -632,7 +632,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>UPDATE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>UPDATE</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Append DELETE rows for reference categories missing from the output
apply_update_flag now also checks the reverse direction: any Category
present in the reference sheet but absent from the earliest date's
output rows gets a new row appended with UploadType=DELETE and
Quantity set to the reference's quantity (e.g. T528B, ref qty 64).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.3.long.xlsx
+++ b/CategorySIPMaintain.7.3.long.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3671,6 +3671,24 @@
         <v>80</v>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>T528B</t>
+        </is>
+      </c>
+      <c r="C181" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="D181" t="n">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Insert DELETE rows right after the earliest date's block, not at the end
Reference-only categories are now appended immediately after the
earliest date's other rows (e.g. right after T523H on 7/4) instead of
at the very end of the sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DphkeLXanAW8ZqwZHK1tS
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.3.long.xlsx
+++ b/CategorySIPMaintain.7.3.long.xlsx
@@ -848,19 +848,19 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T528B</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
-        <v>46208</v>
+        <v>46207</v>
       </c>
       <c r="D24" t="n">
-        <v>850</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25">
@@ -871,14 +871,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D25" t="n">
-        <v>150</v>
+        <v>850</v>
       </c>
     </row>
     <row r="26">
@@ -889,14 +889,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D26" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27">
@@ -907,14 +907,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D27" t="n">
-        <v>84</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28">
@@ -925,14 +925,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D28" t="n">
-        <v>1000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29">
@@ -943,14 +943,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C29" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D29" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="30">
@@ -961,14 +961,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D30" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31">
@@ -979,14 +979,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D31" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="32">
@@ -997,14 +997,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D32" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33">
@@ -1015,14 +1015,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="34">
@@ -1033,14 +1033,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D34" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -1051,14 +1051,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C35" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D35" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36">
@@ -1069,14 +1069,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C36" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D36" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -1087,14 +1087,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C37" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D37" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38">
@@ -1105,14 +1105,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C38" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D38" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39">
@@ -1123,14 +1123,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C39" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D39" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40">
@@ -1141,14 +1141,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C40" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D40" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41">
@@ -1159,14 +1159,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C41" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D41" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42">
@@ -1177,14 +1177,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C42" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D42" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="43">
@@ -1195,14 +1195,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C43" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D43" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44">
@@ -1213,14 +1213,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C44" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D44" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="45">
@@ -1231,14 +1231,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C45" s="1" t="n">
         <v>46208</v>
       </c>
       <c r="D45" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="46">
@@ -1249,14 +1249,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C46" s="1" t="n">
-        <v>46209</v>
+        <v>46208</v>
       </c>
       <c r="D46" t="n">
-        <v>850</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47">
@@ -1267,14 +1267,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C47" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D47" t="n">
-        <v>150</v>
+        <v>850</v>
       </c>
     </row>
     <row r="48">
@@ -1285,14 +1285,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C48" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D48" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49">
@@ -1303,14 +1303,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C49" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D49" t="n">
-        <v>84</v>
+        <v>200</v>
       </c>
     </row>
     <row r="50">
@@ -1321,14 +1321,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C50" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D50" t="n">
-        <v>1000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51">
@@ -1339,14 +1339,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C51" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D51" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="52">
@@ -1357,14 +1357,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C52" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D52" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53">
@@ -1375,14 +1375,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C53" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D53" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="54">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C54" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D54" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C55" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D55" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="56">
@@ -1429,14 +1429,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C56" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D56" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="57">
@@ -1447,14 +1447,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C57" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D57" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58">
@@ -1465,14 +1465,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C58" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D58" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59">
@@ -1483,14 +1483,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C59" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D59" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60">
@@ -1501,14 +1501,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C60" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D60" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="61">
@@ -1519,14 +1519,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C61" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D61" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62">
@@ -1537,14 +1537,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C62" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D62" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63">
@@ -1555,14 +1555,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C63" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D63" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="64">
@@ -1573,14 +1573,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C64" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D64" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="65">
@@ -1591,14 +1591,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C65" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D65" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66">
@@ -1609,14 +1609,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C66" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D66" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="67">
@@ -1627,14 +1627,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C67" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="D67" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="68">
@@ -1645,14 +1645,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C68" s="1" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="D68" t="n">
-        <v>850</v>
+        <v>80</v>
       </c>
     </row>
     <row r="69">
@@ -1663,14 +1663,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C69" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D69" t="n">
-        <v>150</v>
+        <v>850</v>
       </c>
     </row>
     <row r="70">
@@ -1681,14 +1681,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C70" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D70" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
     </row>
     <row r="71">
@@ -1699,14 +1699,14 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C71" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D71" t="n">
-        <v>84</v>
+        <v>250</v>
       </c>
     </row>
     <row r="72">
@@ -1717,14 +1717,14 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C72" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D72" t="n">
-        <v>1050</v>
+        <v>84</v>
       </c>
     </row>
     <row r="73">
@@ -1735,14 +1735,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C73" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D73" t="n">
-        <v>150</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="74">
@@ -1753,14 +1753,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C74" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D74" t="n">
-        <v>66</v>
+        <v>150</v>
       </c>
     </row>
     <row r="75">
@@ -1771,14 +1771,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C75" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D75" t="n">
-        <v>900</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76">
@@ -1789,14 +1789,14 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C76" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D76" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="77">
@@ -1807,14 +1807,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C77" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D77" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="78">
@@ -1825,14 +1825,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C78" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D78" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="79">
@@ -1843,14 +1843,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C79" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D79" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -1861,14 +1861,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C80" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D80" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="81">
@@ -1879,14 +1879,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C81" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D81" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82">
@@ -1897,14 +1897,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C82" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D82" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="83">
@@ -1915,14 +1915,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C83" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D83" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="84">
@@ -1933,14 +1933,14 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C84" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D84" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="85">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C85" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D85" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="86">
@@ -1969,14 +1969,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C86" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D86" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="87">
@@ -1987,14 +1987,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C87" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D87" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="88">
@@ -2005,14 +2005,14 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C88" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D88" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="89">
@@ -2023,14 +2023,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C89" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D89" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="90">
@@ -2041,14 +2041,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C90" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="D90" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="91">
@@ -2059,14 +2059,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C91" s="1" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="D91" t="n">
-        <v>650</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92">
@@ -2077,14 +2077,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C92" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D92" t="n">
-        <v>150</v>
+        <v>650</v>
       </c>
     </row>
     <row r="93">
@@ -2095,14 +2095,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C93" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D93" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
     </row>
     <row r="94">
@@ -2113,14 +2113,14 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B 2</t>
         </is>
       </c>
       <c r="C94" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D94" t="n">
-        <v>350</v>
+        <v>50</v>
       </c>
     </row>
     <row r="95">
@@ -2131,14 +2131,14 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C95" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D95" t="n">
-        <v>84</v>
+        <v>350</v>
       </c>
     </row>
     <row r="96">
@@ -2149,14 +2149,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C96" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D96" t="n">
-        <v>1050</v>
+        <v>84</v>
       </c>
     </row>
     <row r="97">
@@ -2167,14 +2167,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C97" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D97" t="n">
-        <v>150</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="98">
@@ -2185,14 +2185,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C98" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D98" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="99">
@@ -2203,14 +2203,14 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C99" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D99" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="100">
@@ -2221,14 +2221,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C100" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D100" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="101">
@@ -2239,14 +2239,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C101" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D101" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="102">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C102" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D102" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="103">
@@ -2275,14 +2275,14 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C103" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D103" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="104">
@@ -2293,14 +2293,14 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C104" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D104" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105">
@@ -2311,14 +2311,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C105" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D105" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="106">
@@ -2329,14 +2329,14 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C106" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D106" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="107">
@@ -2347,14 +2347,14 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C107" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D107" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="108">
@@ -2365,14 +2365,14 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C108" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D108" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109">
@@ -2383,14 +2383,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C109" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D109" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="110">
@@ -2401,14 +2401,14 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C110" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D110" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="111">
@@ -2419,14 +2419,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C111" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D111" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="112">
@@ -2437,14 +2437,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C112" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D112" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="113">
@@ -2455,14 +2455,14 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C113" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="D113" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="114">
@@ -2473,14 +2473,14 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C114" s="1" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="D114" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="115">
@@ -2491,14 +2491,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C115" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D115" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
     </row>
     <row r="116">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>T59B 2</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C116" s="1" t="n">
@@ -2527,14 +2527,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B 2</t>
         </is>
       </c>
       <c r="C117" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D117" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
     </row>
     <row r="118">
@@ -2545,14 +2545,14 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C118" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D118" t="n">
-        <v>84</v>
+        <v>300</v>
       </c>
     </row>
     <row r="119">
@@ -2563,14 +2563,14 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C119" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D119" t="n">
-        <v>1050</v>
+        <v>84</v>
       </c>
     </row>
     <row r="120">
@@ -2581,14 +2581,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C120" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D120" t="n">
-        <v>150</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="121">
@@ -2599,14 +2599,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C121" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D121" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="122">
@@ -2617,14 +2617,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C122" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D122" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="123">
@@ -2635,14 +2635,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C123" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D123" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="124">
@@ -2653,14 +2653,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C124" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D124" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="125">
@@ -2671,14 +2671,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C125" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D125" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="126">
@@ -2689,14 +2689,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C126" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D126" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="127">
@@ -2707,14 +2707,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C127" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D127" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128">
@@ -2725,14 +2725,14 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C128" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D128" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="129">
@@ -2743,14 +2743,14 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C129" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D129" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="130">
@@ -2761,14 +2761,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C130" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D130" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="131">
@@ -2779,14 +2779,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C131" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D131" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="132">
@@ -2797,14 +2797,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C132" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D132" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="133">
@@ -2815,14 +2815,14 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C133" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D133" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="134">
@@ -2833,14 +2833,14 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C134" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D134" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="135">
@@ -2851,14 +2851,14 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C135" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D135" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="136">
@@ -2869,14 +2869,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C136" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="D136" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="137">
@@ -2887,14 +2887,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C137" s="1" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="D137" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="138">
@@ -2905,14 +2905,14 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C138" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D138" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
     </row>
     <row r="139">
@@ -2923,14 +2923,14 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C139" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D139" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
     </row>
     <row r="140">
@@ -2941,14 +2941,14 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C140" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D140" t="n">
-        <v>84</v>
+        <v>400</v>
       </c>
     </row>
     <row r="141">
@@ -2959,14 +2959,14 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C141" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D141" t="n">
-        <v>1000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="142">
@@ -2977,14 +2977,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C142" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D142" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="143">
@@ -2995,14 +2995,14 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C143" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D143" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="144">
@@ -3013,14 +3013,14 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C144" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D144" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="145">
@@ -3031,14 +3031,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C145" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D145" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="146">
@@ -3049,14 +3049,14 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C146" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D146" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="147">
@@ -3067,14 +3067,14 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C147" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D147" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="148">
@@ -3085,14 +3085,14 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C148" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D148" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="149">
@@ -3103,14 +3103,14 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C149" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D149" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150">
@@ -3121,14 +3121,14 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C150" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D150" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="151">
@@ -3139,14 +3139,14 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C151" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D151" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="152">
@@ -3157,14 +3157,14 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C152" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D152" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="153">
@@ -3175,14 +3175,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C153" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D153" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="154">
@@ -3193,14 +3193,14 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C154" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D154" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="155">
@@ -3211,14 +3211,14 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C155" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D155" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="156">
@@ -3229,14 +3229,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C156" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D156" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="157">
@@ -3247,14 +3247,14 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C157" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D157" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="158">
@@ -3265,14 +3265,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C158" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="D158" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="159">
@@ -3283,14 +3283,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C159" s="1" t="n">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="D159" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="160">
@@ -3301,14 +3301,14 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>T59B</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C160" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D160" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
     </row>
     <row r="161">
@@ -3319,14 +3319,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T59B</t>
         </is>
       </c>
       <c r="C161" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D161" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
     </row>
     <row r="162">
@@ -3337,14 +3337,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Flat T</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C162" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D162" t="n">
-        <v>84</v>
+        <v>400</v>
       </c>
     </row>
     <row r="163">
@@ -3355,14 +3355,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>T-A42</t>
+          <t>Flat T</t>
         </is>
       </c>
       <c r="C163" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D163" t="n">
-        <v>1000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="164">
@@ -3373,14 +3373,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>T-G</t>
+          <t>T-A42</t>
         </is>
       </c>
       <c r="C164" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D164" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="165">
@@ -3391,14 +3391,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T-G</t>
         </is>
       </c>
       <c r="C165" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D165" t="n">
-        <v>900</v>
+        <v>150</v>
       </c>
     </row>
     <row r="166">
@@ -3409,14 +3409,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>1.9V</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C166" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D166" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
     </row>
     <row r="167">
@@ -3427,14 +3427,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2.0V</t>
+          <t>1.9V</t>
         </is>
       </c>
       <c r="C167" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D167" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="168">
@@ -3445,14 +3445,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>2.0V</t>
         </is>
       </c>
       <c r="C168" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D168" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="169">
@@ -3463,14 +3463,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C169" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D169" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="170">
@@ -3481,14 +3481,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C170" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D170" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="171">
@@ -3499,14 +3499,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>T530D 2</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C171" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D171" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172">
@@ -3517,14 +3517,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>T530D 3</t>
+          <t>T530D 2</t>
         </is>
       </c>
       <c r="C172" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D172" t="n">
-        <v>168</v>
+        <v>84</v>
       </c>
     </row>
     <row r="173">
@@ -3535,14 +3535,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>T530X</t>
+          <t>T530D 3</t>
         </is>
       </c>
       <c r="C173" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D173" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="174">
@@ -3553,14 +3553,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>T521X</t>
+          <t>T530X</t>
         </is>
       </c>
       <c r="C174" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D174" t="n">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="175">
@@ -3571,14 +3571,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>T530Y</t>
+          <t>T521X</t>
         </is>
       </c>
       <c r="C175" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D175" t="n">
-        <v>174</v>
+        <v>90</v>
       </c>
     </row>
     <row r="176">
@@ -3589,14 +3589,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>T59D 2</t>
+          <t>T530Y</t>
         </is>
       </c>
       <c r="C176" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D176" t="n">
-        <v>630</v>
+        <v>174</v>
       </c>
     </row>
     <row r="177">
@@ -3607,14 +3607,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>T59D 1</t>
+          <t>T59D 2</t>
         </is>
       </c>
       <c r="C177" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D177" t="n">
-        <v>200</v>
+        <v>630</v>
       </c>
     </row>
     <row r="178">
@@ -3625,14 +3625,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>T59V</t>
+          <t>T59D 1</t>
         </is>
       </c>
       <c r="C178" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D178" t="n">
-        <v>420</v>
+        <v>200</v>
       </c>
     </row>
     <row r="179">
@@ -3643,14 +3643,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>T523W</t>
+          <t>T59V</t>
         </is>
       </c>
       <c r="C179" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D179" t="n">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="180">
@@ -3661,32 +3661,32 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>T523H</t>
+          <t>T523W</t>
         </is>
       </c>
       <c r="C180" s="1" t="n">
         <v>46214</v>
       </c>
       <c r="D180" t="n">
-        <v>80</v>
+        <v>322</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>ADD</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>T528B</t>
+          <t>T523H</t>
         </is>
       </c>
       <c r="C181" s="1" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="D181" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>